<commit_message>
updated project status excel sheet
</commit_message>
<xml_diff>
--- a/review/project_status_tracker_super_long_wave.xlsx
+++ b/review/project_status_tracker_super_long_wave.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yutak\eda\designs\03_super_long_wave\2026_sscs_gf180\review\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3450797-6C22-4842-A14C-ABC69EE30D76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B4C343A-C51D-4AD1-85BC-17947801E36B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="20" windowWidth="19180" windowHeight="11260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="40">
   <si>
     <t>No</t>
     <phoneticPr fontId="1"/>
@@ -63,10 +63,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>Buttercutter</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>Charge pump</t>
     <phoneticPr fontId="1"/>
   </si>
@@ -75,18 +71,10 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>Buffer</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>Project status tracker</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>updated on July 9</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>Main Component</t>
     <phoneticPr fontId="1"/>
   </si>
@@ -157,9 +145,6 @@
   <si>
     <t>Corner simulation</t>
     <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>tb_buffer.sch</t>
   </si>
   <si>
     <t>CP_LF.sch</t>
@@ -178,6 +163,26 @@
   <si>
     <t>Design
 Checklist</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>NAND</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>DFF</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>INVERTER</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>updated on July 17</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Voltage follower</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -243,7 +248,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -292,12 +297,23 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -324,6 +340,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="ハイパーリンク" xfId="1" builtinId="8"/>
@@ -605,7 +622,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="5.75" customWidth="1"/>
@@ -622,12 +639,12 @@
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:14">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:14" s="1" customFormat="1" ht="42" customHeight="1">
@@ -635,10 +652,10 @@
         <v>0</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>1</v>
@@ -647,19 +664,19 @@
         <v>2</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="K3" s="2" t="s">
         <v>4</v>
@@ -678,296 +695,254 @@
       <c r="A4" s="3">
         <v>1</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="4"/>
+      <c r="C4" s="4" t="s">
+        <v>23</v>
+      </c>
       <c r="D4" s="11" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>23</v>
+        <v>18</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>24</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="K4" s="7" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="M4" s="7" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N4" s="7" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:14">
       <c r="A5" s="3">
         <v>2</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="4"/>
+      <c r="B5" s="12"/>
+      <c r="C5" s="4" t="s">
+        <v>35</v>
+      </c>
       <c r="D5" s="11" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="H5" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="J5" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="K5" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="L5" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="M5" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="N5" s="7" t="s">
-        <v>24</v>
-      </c>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="7"/>
+      <c r="K5" s="7"/>
+      <c r="L5" s="7"/>
+      <c r="M5" s="7"/>
+      <c r="N5" s="7"/>
     </row>
     <row r="6" spans="1:14">
       <c r="A6" s="3">
         <v>3</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="4"/>
+      <c r="B6" s="12"/>
+      <c r="C6" s="4" t="s">
+        <v>36</v>
+      </c>
       <c r="D6" s="11" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="H6" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="J6" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="K6" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="L6" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="M6" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="N6" s="7" t="s">
-        <v>24</v>
-      </c>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="7"/>
+      <c r="K6" s="7"/>
+      <c r="L6" s="7"/>
+      <c r="M6" s="7"/>
+      <c r="N6" s="7"/>
     </row>
     <row r="7" spans="1:14">
       <c r="A7" s="3">
         <v>4</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="4"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="4" t="s">
+        <v>37</v>
+      </c>
       <c r="D7" s="11" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="H7" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="I7" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="J7" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="K7" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="L7" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="M7" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="N7" s="7" t="s">
-        <v>24</v>
-      </c>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
+      <c r="L7" s="7"/>
+      <c r="M7" s="7"/>
+      <c r="N7" s="7"/>
     </row>
     <row r="8" spans="1:14">
       <c r="A8" s="3">
         <v>5</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="C8" s="4"/>
       <c r="D8" s="11" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="J8" s="7" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="K8" s="7" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="L8" s="7" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="M8" s="7" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N8" s="7" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:14">
       <c r="A9" s="3">
         <v>6</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" s="4"/>
+      <c r="D9" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F9" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="G9" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="H9" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="D9" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F9" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="G9" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="H9" s="10" t="s">
-        <v>37</v>
-      </c>
       <c r="I9" s="3" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="J9" s="7" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="K9" s="7" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="L9" s="7" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="M9" s="7" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N9" s="7" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:14">
       <c r="A10" s="3">
         <v>7</v>
       </c>
-      <c r="B10" s="9"/>
-      <c r="C10" s="4" t="s">
-        <v>25</v>
-      </c>
+      <c r="B10" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="4"/>
       <c r="D10" s="11" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="G10" s="7" t="s">
-        <v>24</v>
+        <v>20</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>20</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="J10" s="7" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="K10" s="7" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="L10" s="7" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="M10" s="7" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N10" s="7" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11" spans="1:14">
@@ -975,93 +950,246 @@
         <v>8</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="C11" s="4"/>
       <c r="D11" s="11" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="G11" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G11" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="H11" s="3" t="s">
-        <v>31</v>
+      <c r="H11" s="10" t="s">
+        <v>32</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="J11" s="7" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="K11" s="7" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="L11" s="7" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="M11" s="7" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N11" s="7" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:14">
       <c r="A12" s="3">
         <v>9</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C12" s="4"/>
+      <c r="B12" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>23</v>
+      </c>
       <c r="D12" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="E12" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G12" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="H12" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="J12" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K12" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="L12" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="M12" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="N12" s="7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14">
+      <c r="A13" s="3">
+        <v>10</v>
+      </c>
+      <c r="B13" s="12"/>
+      <c r="C13" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G13" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="G12" s="7" t="s">
+      <c r="H13" s="10"/>
+      <c r="I13" s="3"/>
+      <c r="J13" s="7"/>
+      <c r="K13" s="7"/>
+      <c r="L13" s="7"/>
+      <c r="M13" s="7"/>
+      <c r="N13" s="7"/>
+    </row>
+    <row r="14" spans="1:14">
+      <c r="A14" s="3">
+        <v>11</v>
+      </c>
+      <c r="B14" s="9"/>
+      <c r="C14" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G14" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="H12" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="I12" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="J12" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="K12" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="L12" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="M12" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="N12" s="7" t="s">
-        <v>24</v>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="J14" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K14" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="L14" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="M14" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="N14" s="7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14">
+      <c r="A15" s="3">
+        <v>12</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C15" s="4"/>
+      <c r="D15" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="J15" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K15" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="L15" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="M15" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="N15" s="7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14">
+      <c r="A16" s="3">
+        <v>13</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16" s="4"/>
+      <c r="D16" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="J16" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K16" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="L16" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="M16" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="N16" s="7" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>
   <hyperlinks>
-    <hyperlink ref="H7" r:id="rId1" xr:uid="{149FF341-4FB2-4ADA-970F-90D4453931DC}"/>
-    <hyperlink ref="H6" r:id="rId2" xr:uid="{F7D83926-E6F4-4081-87E9-0A1505D2F2BE}"/>
-    <hyperlink ref="H5" r:id="rId3" xr:uid="{E7982A98-110E-492E-8454-44285796A1A5}"/>
-    <hyperlink ref="H8" r:id="rId4" xr:uid="{25C1318D-4904-4F95-83CD-120E2D5AA9DA}"/>
-    <hyperlink ref="H9" r:id="rId5" xr:uid="{7EF73A6F-8A67-4DB9-AB3C-A8742B45A3F0}"/>
+    <hyperlink ref="H9" r:id="rId1" xr:uid="{F7D83926-E6F4-4081-87E9-0A1505D2F2BE}"/>
+    <hyperlink ref="H8" r:id="rId2" xr:uid="{E7982A98-110E-492E-8454-44285796A1A5}"/>
+    <hyperlink ref="H11" r:id="rId3" xr:uid="{25C1318D-4904-4F95-83CD-120E2D5AA9DA}"/>
+    <hyperlink ref="H12" r:id="rId4" xr:uid="{7EF73A6F-8A67-4DB9-AB3C-A8742B45A3F0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>